<commit_message>
Replace 56-62 from accented uppercase to consonant clusters (γγ,σσ,ρχ,φτ,χτ,κτ,νδ)
More useful in everyday Greek speech. Update _wordNums detection and ball colors.

https://claude.ai/code/session_01C4BWLnP7YiAk5ekKacAScz
</commit_message>
<xml_diff>
--- a/kino_mapping_1_80.xlsx
+++ b/kino_mapping_1_80.xlsx
@@ -36,7 +36,7 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="10"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -60,15 +60,15 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00111827"/>
-      <sz val="11"/>
+      <sz val="13"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="00111827"/>
-      <sz val="11"/>
+      <color rgb="00374151"/>
+      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -97,6 +97,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="000891B2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00DC2626"/>
       </patternFill>
     </fill>
@@ -108,26 +113,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001E1B4B"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="4F46E522"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="05966922"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="D9770622"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="DC262622"/>
       </patternFill>
     </fill>
   </fills>
@@ -171,7 +156,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -188,7 +173,10 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -203,13 +191,19 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -218,19 +212,13 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -633,103 +621,108 @@
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>49–62  τονισμένα</t>
+          <t>49–55  τόνοι (ά,έ,ή…)</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
+          <t>56–62  σύμφ. ομάδες (γγ,σσ,ρχ…)</t>
+        </is>
+      </c>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
           <t>63–80  δίψηφα (αι,στ,μπ…)</t>
         </is>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="6" t="n">
+      <c r="A3" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="6" t="n">
+      <c r="B3" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="C3" s="6" t="n">
+      <c r="C3" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="D3" s="6" t="n">
+      <c r="D3" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="E3" s="6" t="n">
+      <c r="E3" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="F3" s="6" t="n">
+      <c r="F3" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="G3" s="6" t="n">
+      <c r="G3" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="H3" s="6" t="n">
+      <c r="H3" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="I3" s="6" t="n">
+      <c r="I3" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="J3" s="6" t="n">
+      <c r="J3" s="7" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="4" ht="38" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>1
 Α</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>2
 Β</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="8" t="inlineStr">
         <is>
           <t>3
 Γ</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="D4" s="8" t="inlineStr">
         <is>
           <t>4
 Δ</t>
         </is>
       </c>
-      <c r="E4" s="7" t="inlineStr">
+      <c r="E4" s="8" t="inlineStr">
         <is>
           <t>5
 Ε</t>
         </is>
       </c>
-      <c r="F4" s="7" t="inlineStr">
+      <c r="F4" s="8" t="inlineStr">
         <is>
           <t>6
 Ζ</t>
         </is>
       </c>
-      <c r="G4" s="7" t="inlineStr">
+      <c r="G4" s="8" t="inlineStr">
         <is>
           <t>7
 Η</t>
         </is>
       </c>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="H4" s="8" t="inlineStr">
         <is>
           <t>8
 Θ</t>
         </is>
       </c>
-      <c r="I4" s="7" t="inlineStr">
+      <c r="I4" s="8" t="inlineStr">
         <is>
           <t>9
 Ι</t>
         </is>
       </c>
-      <c r="J4" s="7" t="inlineStr">
+      <c r="J4" s="8" t="inlineStr">
         <is>
           <t>10
 Κ</t>
@@ -737,61 +730,61 @@
       </c>
     </row>
     <row r="5" ht="38" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>11
 Λ</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>12
 Μ</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>13
 Ν</t>
         </is>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>14
 Ξ</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>15
 Ο</t>
         </is>
       </c>
-      <c r="F5" s="7" t="inlineStr">
+      <c r="F5" s="8" t="inlineStr">
         <is>
           <t>16
 Π</t>
         </is>
       </c>
-      <c r="G5" s="7" t="inlineStr">
+      <c r="G5" s="8" t="inlineStr">
         <is>
           <t>17
 Ρ</t>
         </is>
       </c>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="H5" s="8" t="inlineStr">
         <is>
           <t>18
 Σ</t>
         </is>
       </c>
-      <c r="I5" s="7" t="inlineStr">
+      <c r="I5" s="8" t="inlineStr">
         <is>
           <t>19
 Τ</t>
         </is>
       </c>
-      <c r="J5" s="7" t="inlineStr">
+      <c r="J5" s="8" t="inlineStr">
         <is>
           <t>20
 Υ</t>
@@ -799,61 +792,61 @@
       </c>
     </row>
     <row r="6" ht="38" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>21
 Φ</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>22
 Χ</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>23
 Ψ</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>24
 Ω</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E6" s="9" t="inlineStr">
         <is>
           <t>25
 α</t>
         </is>
       </c>
-      <c r="F6" s="8" t="inlineStr">
+      <c r="F6" s="9" t="inlineStr">
         <is>
           <t>26
 β</t>
         </is>
       </c>
-      <c r="G6" s="8" t="inlineStr">
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>27
 γ</t>
         </is>
       </c>
-      <c r="H6" s="8" t="inlineStr">
+      <c r="H6" s="9" t="inlineStr">
         <is>
           <t>28
 δ</t>
         </is>
       </c>
-      <c r="I6" s="8" t="inlineStr">
+      <c r="I6" s="9" t="inlineStr">
         <is>
           <t>29
 ε</t>
         </is>
       </c>
-      <c r="J6" s="8" t="inlineStr">
+      <c r="J6" s="9" t="inlineStr">
         <is>
           <t>30
 ζ</t>
@@ -861,61 +854,61 @@
       </c>
     </row>
     <row r="7" ht="38" customHeight="1">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>31
 η</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>32
 θ</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>33
 ι</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D7" s="9" t="inlineStr">
         <is>
           <t>34
 κ</t>
         </is>
       </c>
-      <c r="E7" s="8" t="inlineStr">
+      <c r="E7" s="9" t="inlineStr">
         <is>
           <t>35
 λ</t>
         </is>
       </c>
-      <c r="F7" s="8" t="inlineStr">
+      <c r="F7" s="9" t="inlineStr">
         <is>
           <t>36
 μ</t>
         </is>
       </c>
-      <c r="G7" s="8" t="inlineStr">
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>37
 ν</t>
         </is>
       </c>
-      <c r="H7" s="8" t="inlineStr">
+      <c r="H7" s="9" t="inlineStr">
         <is>
           <t>38
 ξ</t>
         </is>
       </c>
-      <c r="I7" s="8" t="inlineStr">
+      <c r="I7" s="9" t="inlineStr">
         <is>
           <t>39
 ο</t>
         </is>
       </c>
-      <c r="J7" s="8" t="inlineStr">
+      <c r="J7" s="9" t="inlineStr">
         <is>
           <t>40
 π</t>
@@ -923,61 +916,61 @@
       </c>
     </row>
     <row r="8" ht="38" customHeight="1">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>41
 ρ</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>42
 σ</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>43
 τ</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="D8" s="9" t="inlineStr">
         <is>
           <t>44
 υ</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="E8" s="9" t="inlineStr">
         <is>
           <t>45
 φ</t>
         </is>
       </c>
-      <c r="F8" s="8" t="inlineStr">
+      <c r="F8" s="9" t="inlineStr">
         <is>
           <t>46
 χ</t>
         </is>
       </c>
-      <c r="G8" s="8" t="inlineStr">
+      <c r="G8" s="9" t="inlineStr">
         <is>
           <t>47
 ψ</t>
         </is>
       </c>
-      <c r="H8" s="8" t="inlineStr">
+      <c r="H8" s="9" t="inlineStr">
         <is>
           <t>48
 ω</t>
         </is>
       </c>
-      <c r="I8" s="9" t="inlineStr">
+      <c r="I8" s="10" t="inlineStr">
         <is>
           <t>49
 ά</t>
         </is>
       </c>
-      <c r="J8" s="9" t="inlineStr">
+      <c r="J8" s="10" t="inlineStr">
         <is>
           <t>50
 έ</t>
@@ -985,123 +978,123 @@
       </c>
     </row>
     <row r="9" ht="38" customHeight="1">
-      <c r="A9" s="9" t="inlineStr">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>51
 ή</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>52
 ί</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="10" t="inlineStr">
         <is>
           <t>53
 ό</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D9" s="10" t="inlineStr">
         <is>
           <t>54
 ύ</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
+      <c r="E9" s="10" t="inlineStr">
         <is>
           <t>55
 ώ</t>
         </is>
       </c>
-      <c r="F9" s="9" t="inlineStr">
+      <c r="F9" s="11" t="inlineStr">
         <is>
           <t>56
-Ά</t>
-        </is>
-      </c>
-      <c r="G9" s="9" t="inlineStr">
+γγ</t>
+        </is>
+      </c>
+      <c r="G9" s="11" t="inlineStr">
         <is>
           <t>57
-Έ</t>
-        </is>
-      </c>
-      <c r="H9" s="9" t="inlineStr">
+σσ</t>
+        </is>
+      </c>
+      <c r="H9" s="11" t="inlineStr">
         <is>
           <t>58
-Ή</t>
-        </is>
-      </c>
-      <c r="I9" s="9" t="inlineStr">
+ρχ</t>
+        </is>
+      </c>
+      <c r="I9" s="11" t="inlineStr">
         <is>
           <t>59
-Ί</t>
-        </is>
-      </c>
-      <c r="J9" s="9" t="inlineStr">
+φτ</t>
+        </is>
+      </c>
+      <c r="J9" s="11" t="inlineStr">
         <is>
           <t>60
-Ό</t>
+χτ</t>
         </is>
       </c>
     </row>
     <row r="10" ht="38" customHeight="1">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>61
-Ύ</t>
-        </is>
-      </c>
-      <c r="B10" s="9" t="inlineStr">
+κτ</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>62
-Ώ</t>
-        </is>
-      </c>
-      <c r="C10" s="10" t="inlineStr">
+νδ</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="inlineStr">
         <is>
           <t>63
 αι</t>
         </is>
       </c>
-      <c r="D10" s="10" t="inlineStr">
+      <c r="D10" s="12" t="inlineStr">
         <is>
           <t>64
 ει</t>
         </is>
       </c>
-      <c r="E10" s="10" t="inlineStr">
+      <c r="E10" s="12" t="inlineStr">
         <is>
           <t>65
 οι</t>
         </is>
       </c>
-      <c r="F10" s="10" t="inlineStr">
+      <c r="F10" s="12" t="inlineStr">
         <is>
           <t>66
 αυ</t>
         </is>
       </c>
-      <c r="G10" s="10" t="inlineStr">
+      <c r="G10" s="12" t="inlineStr">
         <is>
           <t>67
 ευ</t>
         </is>
       </c>
-      <c r="H10" s="10" t="inlineStr">
+      <c r="H10" s="12" t="inlineStr">
         <is>
           <t>68
 ου</t>
         </is>
       </c>
-      <c r="I10" s="10" t="inlineStr">
+      <c r="I10" s="12" t="inlineStr">
         <is>
           <t>69
 μπ</t>
         </is>
       </c>
-      <c r="J10" s="10" t="inlineStr">
+      <c r="J10" s="12" t="inlineStr">
         <is>
           <t>70
 ντ</t>
@@ -1109,61 +1102,61 @@
       </c>
     </row>
     <row r="11" ht="38" customHeight="1">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>71
 γκ</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>72
 τσ</t>
         </is>
       </c>
-      <c r="C11" s="10" t="inlineStr">
+      <c r="C11" s="12" t="inlineStr">
         <is>
           <t>73
 στ</t>
         </is>
       </c>
-      <c r="D11" s="10" t="inlineStr">
+      <c r="D11" s="12" t="inlineStr">
         <is>
           <t>74
 σκ</t>
         </is>
       </c>
-      <c r="E11" s="10" t="inlineStr">
+      <c r="E11" s="12" t="inlineStr">
         <is>
           <t>75
 πρ</t>
         </is>
       </c>
-      <c r="F11" s="10" t="inlineStr">
+      <c r="F11" s="12" t="inlineStr">
         <is>
           <t>76
 τρ</t>
         </is>
       </c>
-      <c r="G11" s="10" t="inlineStr">
+      <c r="G11" s="12" t="inlineStr">
         <is>
           <t>77
 θρ</t>
         </is>
       </c>
-      <c r="H11" s="10" t="inlineStr">
+      <c r="H11" s="12" t="inlineStr">
         <is>
           <t>78
 χρ</t>
         </is>
       </c>
-      <c r="I11" s="10" t="inlineStr">
+      <c r="I11" s="12" t="inlineStr">
         <is>
           <t>79
 σπ</t>
         </is>
       </c>
-      <c r="J11" s="10" t="inlineStr">
+      <c r="J11" s="12" t="inlineStr">
         <is>
           <t>80
 λλ</t>
@@ -1171,12 +1164,13 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
+    <mergeCell ref="G2:H2"/>
     <mergeCell ref="E2:F2"/>
-    <mergeCell ref="G2:J2"/>
+    <mergeCell ref="I2:J2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1191,519 +1185,519 @@
   <dimension ref="A1:D81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t>Αριθμός</t>
         </is>
       </c>
-      <c r="B1" s="11" t="inlineStr">
-        <is>
-          <t>Γράμμα / Δίψηφο</t>
-        </is>
-      </c>
-      <c r="C1" s="11" t="inlineStr">
+      <c r="B1" s="13" t="inlineStr">
+        <is>
+          <t>Σύμβολο</t>
+        </is>
+      </c>
+      <c r="C1" s="13" t="inlineStr">
         <is>
           <t>Κατηγορία</t>
         </is>
       </c>
-      <c r="D1" s="11" t="inlineStr">
-        <is>
-          <t>Περιγραφή</t>
+      <c r="D1" s="13" t="inlineStr">
+        <is>
+          <t>Παράδειγμα</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="12" t="n">
+      <c r="A2" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="13" t="inlineStr">
+      <c r="B2" s="15" t="inlineStr">
         <is>
           <t>Α</t>
         </is>
       </c>
-      <c r="C2" s="13" t="inlineStr">
+      <c r="C2" s="16" t="inlineStr">
         <is>
           <t>ΚΕΦΑΛΑΙΑ</t>
         </is>
       </c>
-      <c r="D2" s="14" t="inlineStr">
-        <is>
-          <t>Κεφαλαία γράμματα ελληνικού αλφαβήτου (Α-Ω)</t>
+      <c r="D2" s="17" t="inlineStr">
+        <is>
+          <t>Α — π.χ. Αλφα</t>
         </is>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="12" t="n">
+      <c r="A3" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B3" s="15" t="inlineStr">
         <is>
           <t>Β</t>
         </is>
       </c>
-      <c r="C3" s="13" t="inlineStr">
+      <c r="C3" s="16" t="inlineStr">
         <is>
           <t>ΚΕΦΑΛΑΙΑ</t>
         </is>
       </c>
-      <c r="D3" s="14" t="inlineStr">
-        <is>
-          <t>Κεφαλαία γράμματα ελληνικού αλφαβήτου (Α-Ω)</t>
+      <c r="D3" s="17" t="inlineStr">
+        <is>
+          <t>Β — π.χ. Βήτα</t>
         </is>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="12" t="n">
+      <c r="A4" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>Γ</t>
         </is>
       </c>
-      <c r="C4" s="13" t="inlineStr">
+      <c r="C4" s="16" t="inlineStr">
         <is>
           <t>ΚΕΦΑΛΑΙΑ</t>
         </is>
       </c>
-      <c r="D4" s="14" t="inlineStr">
-        <is>
-          <t>Κεφαλαία γράμματα ελληνικού αλφαβήτου (Α-Ω)</t>
+      <c r="D4" s="17" t="inlineStr">
+        <is>
+          <t>Γ — π.χ. Γάμα</t>
         </is>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="12" t="n">
+      <c r="A5" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="15" t="inlineStr">
         <is>
           <t>Δ</t>
         </is>
       </c>
-      <c r="C5" s="13" t="inlineStr">
+      <c r="C5" s="16" t="inlineStr">
         <is>
           <t>ΚΕΦΑΛΑΙΑ</t>
         </is>
       </c>
-      <c r="D5" s="14" t="inlineStr">
-        <is>
-          <t>Κεφαλαία γράμματα ελληνικού αλφαβήτου (Α-Ω)</t>
+      <c r="D5" s="17" t="inlineStr">
+        <is>
+          <t>Δ — π.χ. Δέλτα</t>
         </is>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="12" t="n">
+      <c r="A6" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>Ε</t>
         </is>
       </c>
-      <c r="C6" s="13" t="inlineStr">
+      <c r="C6" s="16" t="inlineStr">
         <is>
           <t>ΚΕΦΑΛΑΙΑ</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
-        <is>
-          <t>Κεφαλαία γράμματα ελληνικού αλφαβήτου (Α-Ω)</t>
+      <c r="D6" s="17" t="inlineStr">
+        <is>
+          <t>Ε — π.χ. Έψιλον</t>
         </is>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="12" t="n">
+      <c r="A7" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>Ζ</t>
         </is>
       </c>
-      <c r="C7" s="13" t="inlineStr">
+      <c r="C7" s="16" t="inlineStr">
         <is>
           <t>ΚΕΦΑΛΑΙΑ</t>
         </is>
       </c>
-      <c r="D7" s="14" t="inlineStr">
-        <is>
-          <t>Κεφαλαία γράμματα ελληνικού αλφαβήτου (Α-Ω)</t>
+      <c r="D7" s="17" t="inlineStr">
+        <is>
+          <t>Ζ — π.χ. Ζήτα</t>
         </is>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="12" t="n">
+      <c r="A8" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="15" t="inlineStr">
         <is>
           <t>Η</t>
         </is>
       </c>
-      <c r="C8" s="13" t="inlineStr">
+      <c r="C8" s="16" t="inlineStr">
         <is>
           <t>ΚΕΦΑΛΑΙΑ</t>
         </is>
       </c>
-      <c r="D8" s="14" t="inlineStr">
-        <is>
-          <t>Κεφαλαία γράμματα ελληνικού αλφαβήτου (Α-Ω)</t>
+      <c r="D8" s="17" t="inlineStr">
+        <is>
+          <t>Η — π.χ. Ήτα</t>
         </is>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="12" t="n">
+      <c r="A9" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B9" s="15" t="inlineStr">
         <is>
           <t>Θ</t>
         </is>
       </c>
-      <c r="C9" s="13" t="inlineStr">
+      <c r="C9" s="16" t="inlineStr">
         <is>
           <t>ΚΕΦΑΛΑΙΑ</t>
         </is>
       </c>
-      <c r="D9" s="14" t="inlineStr">
-        <is>
-          <t>Κεφαλαία γράμματα ελληνικού αλφαβήτου (Α-Ω)</t>
+      <c r="D9" s="17" t="inlineStr">
+        <is>
+          <t>Θ — π.χ. Θήτα</t>
         </is>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="12" t="n">
+      <c r="A10" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
         <is>
           <t>Ι</t>
         </is>
       </c>
-      <c r="C10" s="13" t="inlineStr">
+      <c r="C10" s="16" t="inlineStr">
         <is>
           <t>ΚΕΦΑΛΑΙΑ</t>
         </is>
       </c>
-      <c r="D10" s="14" t="inlineStr">
-        <is>
-          <t>Κεφαλαία γράμματα ελληνικού αλφαβήτου (Α-Ω)</t>
+      <c r="D10" s="17" t="inlineStr">
+        <is>
+          <t>Ι — π.χ. Ιώτα</t>
         </is>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="12" t="n">
+      <c r="A11" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B11" s="15" t="inlineStr">
         <is>
           <t>Κ</t>
         </is>
       </c>
-      <c r="C11" s="13" t="inlineStr">
+      <c r="C11" s="16" t="inlineStr">
         <is>
           <t>ΚΕΦΑΛΑΙΑ</t>
         </is>
       </c>
-      <c r="D11" s="14" t="inlineStr">
-        <is>
-          <t>Κεφαλαία γράμματα ελληνικού αλφαβήτου (Α-Ω)</t>
+      <c r="D11" s="17" t="inlineStr">
+        <is>
+          <t>Κ — π.χ. Κάπα</t>
         </is>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="12" t="n">
+      <c r="A12" s="14" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B12" s="15" t="inlineStr">
         <is>
           <t>Λ</t>
         </is>
       </c>
-      <c r="C12" s="13" t="inlineStr">
+      <c r="C12" s="16" t="inlineStr">
         <is>
           <t>ΚΕΦΑΛΑΙΑ</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>Κεφαλαία γράμματα ελληνικού αλφαβήτου (Α-Ω)</t>
+      <c r="D12" s="17" t="inlineStr">
+        <is>
+          <t>Λ — π.χ. Λάμδα</t>
         </is>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="12" t="n">
+      <c r="A13" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="13" t="inlineStr">
+      <c r="B13" s="15" t="inlineStr">
         <is>
           <t>Μ</t>
         </is>
       </c>
-      <c r="C13" s="13" t="inlineStr">
+      <c r="C13" s="16" t="inlineStr">
         <is>
           <t>ΚΕΦΑΛΑΙΑ</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>Κεφαλαία γράμματα ελληνικού αλφαβήτου (Α-Ω)</t>
+      <c r="D13" s="17" t="inlineStr">
+        <is>
+          <t>Μ — π.χ. Μι</t>
         </is>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="12" t="n">
+      <c r="A14" s="14" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="13" t="inlineStr">
+      <c r="B14" s="15" t="inlineStr">
         <is>
           <t>Ν</t>
         </is>
       </c>
-      <c r="C14" s="13" t="inlineStr">
+      <c r="C14" s="16" t="inlineStr">
         <is>
           <t>ΚΕΦΑΛΑΙΑ</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>Κεφαλαία γράμματα ελληνικού αλφαβήτου (Α-Ω)</t>
+      <c r="D14" s="17" t="inlineStr">
+        <is>
+          <t>Ν — π.χ. Νι</t>
         </is>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="12" t="n">
+      <c r="A15" s="14" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B15" s="15" t="inlineStr">
         <is>
           <t>Ξ</t>
         </is>
       </c>
-      <c r="C15" s="13" t="inlineStr">
+      <c r="C15" s="16" t="inlineStr">
         <is>
           <t>ΚΕΦΑΛΑΙΑ</t>
         </is>
       </c>
-      <c r="D15" s="14" t="inlineStr">
-        <is>
-          <t>Κεφαλαία γράμματα ελληνικού αλφαβήτου (Α-Ω)</t>
+      <c r="D15" s="17" t="inlineStr">
+        <is>
+          <t>Ξ — π.χ. Ξι</t>
         </is>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="12" t="n">
+      <c r="A16" s="14" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="13" t="inlineStr">
+      <c r="B16" s="15" t="inlineStr">
         <is>
           <t>Ο</t>
         </is>
       </c>
-      <c r="C16" s="13" t="inlineStr">
+      <c r="C16" s="16" t="inlineStr">
         <is>
           <t>ΚΕΦΑΛΑΙΑ</t>
         </is>
       </c>
-      <c r="D16" s="14" t="inlineStr">
-        <is>
-          <t>Κεφαλαία γράμματα ελληνικού αλφαβήτου (Α-Ω)</t>
+      <c r="D16" s="17" t="inlineStr">
+        <is>
+          <t>Ο — π.χ. Όμικρον</t>
         </is>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="12" t="n">
+      <c r="A17" s="14" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="13" t="inlineStr">
+      <c r="B17" s="15" t="inlineStr">
         <is>
           <t>Π</t>
         </is>
       </c>
-      <c r="C17" s="13" t="inlineStr">
+      <c r="C17" s="16" t="inlineStr">
         <is>
           <t>ΚΕΦΑΛΑΙΑ</t>
         </is>
       </c>
-      <c r="D17" s="14" t="inlineStr">
-        <is>
-          <t>Κεφαλαία γράμματα ελληνικού αλφαβήτου (Α-Ω)</t>
+      <c r="D17" s="17" t="inlineStr">
+        <is>
+          <t>Π — π.χ. Πι</t>
         </is>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="12" t="n">
+      <c r="A18" s="14" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="13" t="inlineStr">
+      <c r="B18" s="15" t="inlineStr">
         <is>
           <t>Ρ</t>
         </is>
       </c>
-      <c r="C18" s="13" t="inlineStr">
+      <c r="C18" s="16" t="inlineStr">
         <is>
           <t>ΚΕΦΑΛΑΙΑ</t>
         </is>
       </c>
-      <c r="D18" s="14" t="inlineStr">
-        <is>
-          <t>Κεφαλαία γράμματα ελληνικού αλφαβήτου (Α-Ω)</t>
+      <c r="D18" s="17" t="inlineStr">
+        <is>
+          <t>Ρ — π.χ. Ρω</t>
         </is>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="12" t="n">
+      <c r="A19" s="14" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="13" t="inlineStr">
+      <c r="B19" s="15" t="inlineStr">
         <is>
           <t>Σ</t>
         </is>
       </c>
-      <c r="C19" s="13" t="inlineStr">
+      <c r="C19" s="16" t="inlineStr">
         <is>
           <t>ΚΕΦΑΛΑΙΑ</t>
         </is>
       </c>
-      <c r="D19" s="14" t="inlineStr">
-        <is>
-          <t>Κεφαλαία γράμματα ελληνικού αλφαβήτου (Α-Ω)</t>
+      <c r="D19" s="17" t="inlineStr">
+        <is>
+          <t>Σ — π.χ. Σίγμα</t>
         </is>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="12" t="n">
+      <c r="A20" s="14" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="13" t="inlineStr">
+      <c r="B20" s="15" t="inlineStr">
         <is>
           <t>Τ</t>
         </is>
       </c>
-      <c r="C20" s="13" t="inlineStr">
+      <c r="C20" s="16" t="inlineStr">
         <is>
           <t>ΚΕΦΑΛΑΙΑ</t>
         </is>
       </c>
-      <c r="D20" s="14" t="inlineStr">
-        <is>
-          <t>Κεφαλαία γράμματα ελληνικού αλφαβήτου (Α-Ω)</t>
+      <c r="D20" s="17" t="inlineStr">
+        <is>
+          <t>Τ — π.χ. Ταυ</t>
         </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="12" t="n">
+      <c r="A21" s="14" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="13" t="inlineStr">
+      <c r="B21" s="15" t="inlineStr">
         <is>
           <t>Υ</t>
         </is>
       </c>
-      <c r="C21" s="13" t="inlineStr">
+      <c r="C21" s="16" t="inlineStr">
         <is>
           <t>ΚΕΦΑΛΑΙΑ</t>
         </is>
       </c>
-      <c r="D21" s="14" t="inlineStr">
-        <is>
-          <t>Κεφαλαία γράμματα ελληνικού αλφαβήτου (Α-Ω)</t>
+      <c r="D21" s="17" t="inlineStr">
+        <is>
+          <t>Υ — π.χ. Ύψιλον</t>
         </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="12" t="n">
+      <c r="A22" s="14" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="13" t="inlineStr">
+      <c r="B22" s="15" t="inlineStr">
         <is>
           <t>Φ</t>
         </is>
       </c>
-      <c r="C22" s="13" t="inlineStr">
+      <c r="C22" s="16" t="inlineStr">
         <is>
           <t>ΚΕΦΑΛΑΙΑ</t>
         </is>
       </c>
-      <c r="D22" s="14" t="inlineStr">
-        <is>
-          <t>Κεφαλαία γράμματα ελληνικού αλφαβήτου (Α-Ω)</t>
+      <c r="D22" s="17" t="inlineStr">
+        <is>
+          <t>Φ — π.χ. Φι</t>
         </is>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="12" t="n">
+      <c r="A23" s="14" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="13" t="inlineStr">
+      <c r="B23" s="15" t="inlineStr">
         <is>
           <t>Χ</t>
         </is>
       </c>
-      <c r="C23" s="13" t="inlineStr">
+      <c r="C23" s="16" t="inlineStr">
         <is>
           <t>ΚΕΦΑΛΑΙΑ</t>
         </is>
       </c>
-      <c r="D23" s="14" t="inlineStr">
-        <is>
-          <t>Κεφαλαία γράμματα ελληνικού αλφαβήτου (Α-Ω)</t>
+      <c r="D23" s="17" t="inlineStr">
+        <is>
+          <t>Χ — π.χ. Χι</t>
         </is>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="12" t="n">
+      <c r="A24" s="14" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="13" t="inlineStr">
+      <c r="B24" s="15" t="inlineStr">
         <is>
           <t>Ψ</t>
         </is>
       </c>
-      <c r="C24" s="13" t="inlineStr">
+      <c r="C24" s="16" t="inlineStr">
         <is>
           <t>ΚΕΦΑΛΑΙΑ</t>
         </is>
       </c>
-      <c r="D24" s="14" t="inlineStr">
-        <is>
-          <t>Κεφαλαία γράμματα ελληνικού αλφαβήτου (Α-Ω)</t>
+      <c r="D24" s="17" t="inlineStr">
+        <is>
+          <t>Ψ — π.χ. Ψι</t>
         </is>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="12" t="n">
+      <c r="A25" s="14" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="13" t="inlineStr">
+      <c r="B25" s="15" t="inlineStr">
         <is>
           <t>Ω</t>
         </is>
       </c>
-      <c r="C25" s="13" t="inlineStr">
+      <c r="C25" s="16" t="inlineStr">
         <is>
           <t>ΚΕΦΑΛΑΙΑ</t>
         </is>
       </c>
-      <c r="D25" s="14" t="inlineStr">
-        <is>
-          <t>Κεφαλαία γράμματα ελληνικού αλφαβήτου (Α-Ω)</t>
+      <c r="D25" s="17" t="inlineStr">
+        <is>
+          <t>Ω — π.χ. Ωμέγα</t>
         </is>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="15" t="n">
+      <c r="A26" s="18" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="16" t="inlineStr">
+      <c r="B26" s="15" t="inlineStr">
         <is>
           <t>α</t>
         </is>
@@ -1713,17 +1707,17 @@
           <t>μικρά</t>
         </is>
       </c>
-      <c r="D26" s="14" t="inlineStr">
-        <is>
-          <t>Πεζά γράμματα ελληνικού αλφαβήτου (α-ω)</t>
+      <c r="D26" s="17" t="inlineStr">
+        <is>
+          <t>α — π.χ. αλφα</t>
         </is>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="15" t="n">
+      <c r="A27" s="18" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="16" t="inlineStr">
+      <c r="B27" s="15" t="inlineStr">
         <is>
           <t>β</t>
         </is>
@@ -1733,17 +1727,17 @@
           <t>μικρά</t>
         </is>
       </c>
-      <c r="D27" s="14" t="inlineStr">
-        <is>
-          <t>Πεζά γράμματα ελληνικού αλφαβήτου (α-ω)</t>
+      <c r="D27" s="17" t="inlineStr">
+        <is>
+          <t>β — π.χ. βήτα</t>
         </is>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="15" t="n">
+      <c r="A28" s="18" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="16" t="inlineStr">
+      <c r="B28" s="15" t="inlineStr">
         <is>
           <t>γ</t>
         </is>
@@ -1753,17 +1747,17 @@
           <t>μικρά</t>
         </is>
       </c>
-      <c r="D28" s="14" t="inlineStr">
-        <is>
-          <t>Πεζά γράμματα ελληνικού αλφαβήτου (α-ω)</t>
+      <c r="D28" s="17" t="inlineStr">
+        <is>
+          <t>γ — π.χ. γάμα</t>
         </is>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="15" t="n">
+      <c r="A29" s="18" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="16" t="inlineStr">
+      <c r="B29" s="15" t="inlineStr">
         <is>
           <t>δ</t>
         </is>
@@ -1773,17 +1767,17 @@
           <t>μικρά</t>
         </is>
       </c>
-      <c r="D29" s="14" t="inlineStr">
-        <is>
-          <t>Πεζά γράμματα ελληνικού αλφαβήτου (α-ω)</t>
+      <c r="D29" s="17" t="inlineStr">
+        <is>
+          <t>δ — π.χ. δέλτα</t>
         </is>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="15" t="n">
+      <c r="A30" s="18" t="n">
         <v>29</v>
       </c>
-      <c r="B30" s="16" t="inlineStr">
+      <c r="B30" s="15" t="inlineStr">
         <is>
           <t>ε</t>
         </is>
@@ -1793,17 +1787,17 @@
           <t>μικρά</t>
         </is>
       </c>
-      <c r="D30" s="14" t="inlineStr">
-        <is>
-          <t>Πεζά γράμματα ελληνικού αλφαβήτου (α-ω)</t>
+      <c r="D30" s="17" t="inlineStr">
+        <is>
+          <t>ε — π.χ. έψιλον</t>
         </is>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="15" t="n">
+      <c r="A31" s="18" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="16" t="inlineStr">
+      <c r="B31" s="15" t="inlineStr">
         <is>
           <t>ζ</t>
         </is>
@@ -1813,17 +1807,17 @@
           <t>μικρά</t>
         </is>
       </c>
-      <c r="D31" s="14" t="inlineStr">
-        <is>
-          <t>Πεζά γράμματα ελληνικού αλφαβήτου (α-ω)</t>
+      <c r="D31" s="17" t="inlineStr">
+        <is>
+          <t>ζ — π.χ. ζήτα</t>
         </is>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="15" t="n">
+      <c r="A32" s="18" t="n">
         <v>31</v>
       </c>
-      <c r="B32" s="16" t="inlineStr">
+      <c r="B32" s="15" t="inlineStr">
         <is>
           <t>η</t>
         </is>
@@ -1833,17 +1827,17 @@
           <t>μικρά</t>
         </is>
       </c>
-      <c r="D32" s="14" t="inlineStr">
-        <is>
-          <t>Πεζά γράμματα ελληνικού αλφαβήτου (α-ω)</t>
+      <c r="D32" s="17" t="inlineStr">
+        <is>
+          <t>η — π.χ. ήτα</t>
         </is>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="15" t="n">
+      <c r="A33" s="18" t="n">
         <v>32</v>
       </c>
-      <c r="B33" s="16" t="inlineStr">
+      <c r="B33" s="15" t="inlineStr">
         <is>
           <t>θ</t>
         </is>
@@ -1853,17 +1847,17 @@
           <t>μικρά</t>
         </is>
       </c>
-      <c r="D33" s="14" t="inlineStr">
-        <is>
-          <t>Πεζά γράμματα ελληνικού αλφαβήτου (α-ω)</t>
+      <c r="D33" s="17" t="inlineStr">
+        <is>
+          <t>θ — π.χ. θήτα</t>
         </is>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="15" t="n">
+      <c r="A34" s="18" t="n">
         <v>33</v>
       </c>
-      <c r="B34" s="16" t="inlineStr">
+      <c r="B34" s="15" t="inlineStr">
         <is>
           <t>ι</t>
         </is>
@@ -1873,17 +1867,17 @@
           <t>μικρά</t>
         </is>
       </c>
-      <c r="D34" s="14" t="inlineStr">
-        <is>
-          <t>Πεζά γράμματα ελληνικού αλφαβήτου (α-ω)</t>
+      <c r="D34" s="17" t="inlineStr">
+        <is>
+          <t>ι — π.χ. ιώτα</t>
         </is>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="15" t="n">
+      <c r="A35" s="18" t="n">
         <v>34</v>
       </c>
-      <c r="B35" s="16" t="inlineStr">
+      <c r="B35" s="15" t="inlineStr">
         <is>
           <t>κ</t>
         </is>
@@ -1893,17 +1887,17 @@
           <t>μικρά</t>
         </is>
       </c>
-      <c r="D35" s="14" t="inlineStr">
-        <is>
-          <t>Πεζά γράμματα ελληνικού αλφαβήτου (α-ω)</t>
+      <c r="D35" s="17" t="inlineStr">
+        <is>
+          <t>κ — π.χ. κάπα</t>
         </is>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="15" t="n">
+      <c r="A36" s="18" t="n">
         <v>35</v>
       </c>
-      <c r="B36" s="16" t="inlineStr">
+      <c r="B36" s="15" t="inlineStr">
         <is>
           <t>λ</t>
         </is>
@@ -1913,17 +1907,17 @@
           <t>μικρά</t>
         </is>
       </c>
-      <c r="D36" s="14" t="inlineStr">
-        <is>
-          <t>Πεζά γράμματα ελληνικού αλφαβήτου (α-ω)</t>
+      <c r="D36" s="17" t="inlineStr">
+        <is>
+          <t>λ — π.χ. λάμδα</t>
         </is>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="15" t="n">
+      <c r="A37" s="18" t="n">
         <v>36</v>
       </c>
-      <c r="B37" s="16" t="inlineStr">
+      <c r="B37" s="15" t="inlineStr">
         <is>
           <t>μ</t>
         </is>
@@ -1933,17 +1927,17 @@
           <t>μικρά</t>
         </is>
       </c>
-      <c r="D37" s="14" t="inlineStr">
-        <is>
-          <t>Πεζά γράμματα ελληνικού αλφαβήτου (α-ω)</t>
+      <c r="D37" s="17" t="inlineStr">
+        <is>
+          <t>μ — π.χ. μι</t>
         </is>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="15" t="n">
+      <c r="A38" s="18" t="n">
         <v>37</v>
       </c>
-      <c r="B38" s="16" t="inlineStr">
+      <c r="B38" s="15" t="inlineStr">
         <is>
           <t>ν</t>
         </is>
@@ -1953,17 +1947,17 @@
           <t>μικρά</t>
         </is>
       </c>
-      <c r="D38" s="14" t="inlineStr">
-        <is>
-          <t>Πεζά γράμματα ελληνικού αλφαβήτου (α-ω)</t>
+      <c r="D38" s="17" t="inlineStr">
+        <is>
+          <t>ν — π.χ. νι</t>
         </is>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="15" t="n">
+      <c r="A39" s="18" t="n">
         <v>38</v>
       </c>
-      <c r="B39" s="16" t="inlineStr">
+      <c r="B39" s="15" t="inlineStr">
         <is>
           <t>ξ</t>
         </is>
@@ -1973,17 +1967,17 @@
           <t>μικρά</t>
         </is>
       </c>
-      <c r="D39" s="14" t="inlineStr">
-        <is>
-          <t>Πεζά γράμματα ελληνικού αλφαβήτου (α-ω)</t>
+      <c r="D39" s="17" t="inlineStr">
+        <is>
+          <t>ξ — π.χ. ξι</t>
         </is>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="15" t="n">
+      <c r="A40" s="18" t="n">
         <v>39</v>
       </c>
-      <c r="B40" s="16" t="inlineStr">
+      <c r="B40" s="15" t="inlineStr">
         <is>
           <t>ο</t>
         </is>
@@ -1993,17 +1987,17 @@
           <t>μικρά</t>
         </is>
       </c>
-      <c r="D40" s="14" t="inlineStr">
-        <is>
-          <t>Πεζά γράμματα ελληνικού αλφαβήτου (α-ω)</t>
+      <c r="D40" s="17" t="inlineStr">
+        <is>
+          <t>ο — π.χ. όμικρον</t>
         </is>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="15" t="n">
+      <c r="A41" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="B41" s="16" t="inlineStr">
+      <c r="B41" s="15" t="inlineStr">
         <is>
           <t>π</t>
         </is>
@@ -2013,17 +2007,17 @@
           <t>μικρά</t>
         </is>
       </c>
-      <c r="D41" s="14" t="inlineStr">
-        <is>
-          <t>Πεζά γράμματα ελληνικού αλφαβήτου (α-ω)</t>
+      <c r="D41" s="17" t="inlineStr">
+        <is>
+          <t>π — π.χ. πι</t>
         </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="15" t="n">
+      <c r="A42" s="18" t="n">
         <v>41</v>
       </c>
-      <c r="B42" s="16" t="inlineStr">
+      <c r="B42" s="15" t="inlineStr">
         <is>
           <t>ρ</t>
         </is>
@@ -2033,17 +2027,17 @@
           <t>μικρά</t>
         </is>
       </c>
-      <c r="D42" s="14" t="inlineStr">
-        <is>
-          <t>Πεζά γράμματα ελληνικού αλφαβήτου (α-ω)</t>
+      <c r="D42" s="17" t="inlineStr">
+        <is>
+          <t>ρ — π.χ. ρω</t>
         </is>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="15" t="n">
+      <c r="A43" s="18" t="n">
         <v>42</v>
       </c>
-      <c r="B43" s="16" t="inlineStr">
+      <c r="B43" s="15" t="inlineStr">
         <is>
           <t>σ</t>
         </is>
@@ -2053,17 +2047,17 @@
           <t>μικρά</t>
         </is>
       </c>
-      <c r="D43" s="14" t="inlineStr">
-        <is>
-          <t>Πεζά γράμματα ελληνικού αλφαβήτου (α-ω)</t>
+      <c r="D43" s="17" t="inlineStr">
+        <is>
+          <t>σ — π.χ. σίγμα</t>
         </is>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="15" t="n">
+      <c r="A44" s="18" t="n">
         <v>43</v>
       </c>
-      <c r="B44" s="16" t="inlineStr">
+      <c r="B44" s="15" t="inlineStr">
         <is>
           <t>τ</t>
         </is>
@@ -2073,17 +2067,17 @@
           <t>μικρά</t>
         </is>
       </c>
-      <c r="D44" s="14" t="inlineStr">
-        <is>
-          <t>Πεζά γράμματα ελληνικού αλφαβήτου (α-ω)</t>
+      <c r="D44" s="17" t="inlineStr">
+        <is>
+          <t>τ — π.χ. ταυ</t>
         </is>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
-      <c r="A45" s="15" t="n">
+      <c r="A45" s="18" t="n">
         <v>44</v>
       </c>
-      <c r="B45" s="16" t="inlineStr">
+      <c r="B45" s="15" t="inlineStr">
         <is>
           <t>υ</t>
         </is>
@@ -2093,17 +2087,17 @@
           <t>μικρά</t>
         </is>
       </c>
-      <c r="D45" s="14" t="inlineStr">
-        <is>
-          <t>Πεζά γράμματα ελληνικού αλφαβήτου (α-ω)</t>
+      <c r="D45" s="17" t="inlineStr">
+        <is>
+          <t>υ — π.χ. ύψιλον</t>
         </is>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
-      <c r="A46" s="15" t="n">
+      <c r="A46" s="18" t="n">
         <v>45</v>
       </c>
-      <c r="B46" s="16" t="inlineStr">
+      <c r="B46" s="15" t="inlineStr">
         <is>
           <t>φ</t>
         </is>
@@ -2113,17 +2107,17 @@
           <t>μικρά</t>
         </is>
       </c>
-      <c r="D46" s="14" t="inlineStr">
-        <is>
-          <t>Πεζά γράμματα ελληνικού αλφαβήτου (α-ω)</t>
+      <c r="D46" s="17" t="inlineStr">
+        <is>
+          <t>φ — π.χ. φι</t>
         </is>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="15" t="n">
+      <c r="A47" s="18" t="n">
         <v>46</v>
       </c>
-      <c r="B47" s="16" t="inlineStr">
+      <c r="B47" s="15" t="inlineStr">
         <is>
           <t>χ</t>
         </is>
@@ -2133,17 +2127,17 @@
           <t>μικρά</t>
         </is>
       </c>
-      <c r="D47" s="14" t="inlineStr">
-        <is>
-          <t>Πεζά γράμματα ελληνικού αλφαβήτου (α-ω)</t>
+      <c r="D47" s="17" t="inlineStr">
+        <is>
+          <t>χ — π.χ. χι</t>
         </is>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="15" t="n">
+      <c r="A48" s="18" t="n">
         <v>47</v>
       </c>
-      <c r="B48" s="16" t="inlineStr">
+      <c r="B48" s="15" t="inlineStr">
         <is>
           <t>ψ</t>
         </is>
@@ -2153,17 +2147,17 @@
           <t>μικρά</t>
         </is>
       </c>
-      <c r="D48" s="14" t="inlineStr">
-        <is>
-          <t>Πεζά γράμματα ελληνικού αλφαβήτου (α-ω)</t>
+      <c r="D48" s="17" t="inlineStr">
+        <is>
+          <t>ψ — π.χ. ψι</t>
         </is>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
-      <c r="A49" s="15" t="n">
+      <c r="A49" s="18" t="n">
         <v>48</v>
       </c>
-      <c r="B49" s="16" t="inlineStr">
+      <c r="B49" s="15" t="inlineStr">
         <is>
           <t>ω</t>
         </is>
@@ -2173,649 +2167,649 @@
           <t>μικρά</t>
         </is>
       </c>
-      <c r="D49" s="14" t="inlineStr">
-        <is>
-          <t>Πεζά γράμματα ελληνικού αλφαβήτου (α-ω)</t>
+      <c r="D49" s="17" t="inlineStr">
+        <is>
+          <t>ω — π.χ. ωμέγα</t>
         </is>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
-      <c r="A50" s="17" t="n">
+      <c r="A50" s="19" t="n">
         <v>49</v>
       </c>
-      <c r="B50" s="18" t="inlineStr">
+      <c r="B50" s="15" t="inlineStr">
         <is>
           <t>ά</t>
         </is>
       </c>
-      <c r="C50" s="18" t="inlineStr">
-        <is>
-          <t>τόνοι μικρά</t>
-        </is>
-      </c>
-      <c r="D50" s="14" t="inlineStr">
-        <is>
-          <t>Τονισμένα πεζά φωνήεντα (ά,έ,ή,ί,ό,ύ,ώ)</t>
+      <c r="C50" s="16" t="inlineStr">
+        <is>
+          <t>τόνοι</t>
+        </is>
+      </c>
+      <c r="D50" s="17" t="inlineStr">
+        <is>
+          <t>ά — π.χ. άντρας</t>
         </is>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
-      <c r="A51" s="17" t="n">
+      <c r="A51" s="19" t="n">
         <v>50</v>
       </c>
-      <c r="B51" s="18" t="inlineStr">
+      <c r="B51" s="15" t="inlineStr">
         <is>
           <t>έ</t>
         </is>
       </c>
-      <c r="C51" s="18" t="inlineStr">
-        <is>
-          <t>τόνοι μικρά</t>
-        </is>
-      </c>
-      <c r="D51" s="14" t="inlineStr">
-        <is>
-          <t>Τονισμένα πεζά φωνήεντα (ά,έ,ή,ί,ό,ύ,ώ)</t>
+      <c r="C51" s="16" t="inlineStr">
+        <is>
+          <t>τόνοι</t>
+        </is>
+      </c>
+      <c r="D51" s="17" t="inlineStr">
+        <is>
+          <t>έ — π.χ. έγγραφο</t>
         </is>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
-      <c r="A52" s="17" t="n">
+      <c r="A52" s="19" t="n">
         <v>51</v>
       </c>
-      <c r="B52" s="18" t="inlineStr">
+      <c r="B52" s="15" t="inlineStr">
         <is>
           <t>ή</t>
         </is>
       </c>
-      <c r="C52" s="18" t="inlineStr">
-        <is>
-          <t>τόνοι μικρά</t>
-        </is>
-      </c>
-      <c r="D52" s="14" t="inlineStr">
-        <is>
-          <t>Τονισμένα πεζά φωνήεντα (ά,έ,ή,ί,ό,ύ,ώ)</t>
+      <c r="C52" s="16" t="inlineStr">
+        <is>
+          <t>τόνοι</t>
+        </is>
+      </c>
+      <c r="D52" s="17" t="inlineStr">
+        <is>
+          <t>ή — π.χ. ήλιος</t>
         </is>
       </c>
     </row>
     <row r="53" ht="18" customHeight="1">
-      <c r="A53" s="17" t="n">
+      <c r="A53" s="19" t="n">
         <v>52</v>
       </c>
-      <c r="B53" s="18" t="inlineStr">
+      <c r="B53" s="15" t="inlineStr">
         <is>
           <t>ί</t>
         </is>
       </c>
-      <c r="C53" s="18" t="inlineStr">
-        <is>
-          <t>τόνοι μικρά</t>
-        </is>
-      </c>
-      <c r="D53" s="14" t="inlineStr">
-        <is>
-          <t>Τονισμένα πεζά φωνήεντα (ά,έ,ή,ί,ό,ύ,ώ)</t>
+      <c r="C53" s="16" t="inlineStr">
+        <is>
+          <t>τόνοι</t>
+        </is>
+      </c>
+      <c r="D53" s="17" t="inlineStr">
+        <is>
+          <t>ί — π.χ. ίδιος</t>
         </is>
       </c>
     </row>
     <row r="54" ht="18" customHeight="1">
-      <c r="A54" s="17" t="n">
+      <c r="A54" s="19" t="n">
         <v>53</v>
       </c>
-      <c r="B54" s="18" t="inlineStr">
+      <c r="B54" s="15" t="inlineStr">
         <is>
           <t>ό</t>
         </is>
       </c>
-      <c r="C54" s="18" t="inlineStr">
-        <is>
-          <t>τόνοι μικρά</t>
-        </is>
-      </c>
-      <c r="D54" s="14" t="inlineStr">
-        <is>
-          <t>Τονισμένα πεζά φωνήεντα (ά,έ,ή,ί,ό,ύ,ώ)</t>
+      <c r="C54" s="16" t="inlineStr">
+        <is>
+          <t>τόνοι</t>
+        </is>
+      </c>
+      <c r="D54" s="17" t="inlineStr">
+        <is>
+          <t>ό — π.χ. όνομα</t>
         </is>
       </c>
     </row>
     <row r="55" ht="18" customHeight="1">
-      <c r="A55" s="17" t="n">
+      <c r="A55" s="19" t="n">
         <v>54</v>
       </c>
-      <c r="B55" s="18" t="inlineStr">
+      <c r="B55" s="15" t="inlineStr">
         <is>
           <t>ύ</t>
         </is>
       </c>
-      <c r="C55" s="18" t="inlineStr">
-        <is>
-          <t>τόνοι μικρά</t>
-        </is>
-      </c>
-      <c r="D55" s="14" t="inlineStr">
-        <is>
-          <t>Τονισμένα πεζά φωνήεντα (ά,έ,ή,ί,ό,ύ,ώ)</t>
+      <c r="C55" s="16" t="inlineStr">
+        <is>
+          <t>τόνοι</t>
+        </is>
+      </c>
+      <c r="D55" s="17" t="inlineStr">
+        <is>
+          <t>ύ — π.χ. ύπνος</t>
         </is>
       </c>
     </row>
     <row r="56" ht="18" customHeight="1">
-      <c r="A56" s="17" t="n">
+      <c r="A56" s="19" t="n">
         <v>55</v>
       </c>
-      <c r="B56" s="18" t="inlineStr">
+      <c r="B56" s="15" t="inlineStr">
         <is>
           <t>ώ</t>
         </is>
       </c>
-      <c r="C56" s="18" t="inlineStr">
-        <is>
-          <t>τόνοι μικρά</t>
-        </is>
-      </c>
-      <c r="D56" s="14" t="inlineStr">
-        <is>
-          <t>Τονισμένα πεζά φωνήεντα (ά,έ,ή,ί,ό,ύ,ώ)</t>
+      <c r="C56" s="16" t="inlineStr">
+        <is>
+          <t>τόνοι</t>
+        </is>
+      </c>
+      <c r="D56" s="17" t="inlineStr">
+        <is>
+          <t>ώ — π.χ. ώρα</t>
         </is>
       </c>
     </row>
     <row r="57" ht="18" customHeight="1">
-      <c r="A57" s="17" t="n">
+      <c r="A57" s="20" t="n">
         <v>56</v>
       </c>
-      <c r="B57" s="18" t="inlineStr">
-        <is>
-          <t>Ά</t>
-        </is>
-      </c>
-      <c r="C57" s="18" t="inlineStr">
-        <is>
-          <t>τόνοι κεφ.</t>
-        </is>
-      </c>
-      <c r="D57" s="14" t="inlineStr">
-        <is>
-          <t>Τονισμένα κεφαλαία φωνήεντα (Ά,Έ,Ή,Ί,Ό,Ύ,Ώ)</t>
+      <c r="B57" s="15" t="inlineStr">
+        <is>
+          <t>γγ</t>
+        </is>
+      </c>
+      <c r="C57" s="16" t="inlineStr">
+        <is>
+          <t>συμφωνικές ομάδες</t>
+        </is>
+      </c>
+      <c r="D57" s="17" t="inlineStr">
+        <is>
+          <t>γγ — π.χ. άγγελος, εγγύς</t>
         </is>
       </c>
     </row>
     <row r="58" ht="18" customHeight="1">
-      <c r="A58" s="17" t="n">
+      <c r="A58" s="20" t="n">
         <v>57</v>
       </c>
-      <c r="B58" s="18" t="inlineStr">
-        <is>
-          <t>Έ</t>
-        </is>
-      </c>
-      <c r="C58" s="18" t="inlineStr">
-        <is>
-          <t>τόνοι κεφ.</t>
-        </is>
-      </c>
-      <c r="D58" s="14" t="inlineStr">
-        <is>
-          <t>Τονισμένα κεφαλαία φωνήεντα (Ά,Έ,Ή,Ί,Ό,Ύ,Ώ)</t>
+      <c r="B58" s="15" t="inlineStr">
+        <is>
+          <t>σσ</t>
+        </is>
+      </c>
+      <c r="C58" s="16" t="inlineStr">
+        <is>
+          <t>συμφωνικές ομάδες</t>
+        </is>
+      </c>
+      <c r="D58" s="17" t="inlineStr">
+        <is>
+          <t>σσ — π.χ. θάλασσα, γλώσσα</t>
         </is>
       </c>
     </row>
     <row r="59" ht="18" customHeight="1">
-      <c r="A59" s="17" t="n">
+      <c r="A59" s="20" t="n">
         <v>58</v>
       </c>
-      <c r="B59" s="18" t="inlineStr">
-        <is>
-          <t>Ή</t>
-        </is>
-      </c>
-      <c r="C59" s="18" t="inlineStr">
-        <is>
-          <t>τόνοι κεφ.</t>
-        </is>
-      </c>
-      <c r="D59" s="14" t="inlineStr">
-        <is>
-          <t>Τονισμένα κεφαλαία φωνήεντα (Ά,Έ,Ή,Ί,Ό,Ύ,Ώ)</t>
+      <c r="B59" s="15" t="inlineStr">
+        <is>
+          <t>ρχ</t>
+        </is>
+      </c>
+      <c r="C59" s="16" t="inlineStr">
+        <is>
+          <t>συμφωνικές ομάδες</t>
+        </is>
+      </c>
+      <c r="D59" s="17" t="inlineStr">
+        <is>
+          <t>ρχ — π.χ. αρχή, πατριάρχης</t>
         </is>
       </c>
     </row>
     <row r="60" ht="18" customHeight="1">
-      <c r="A60" s="17" t="n">
+      <c r="A60" s="20" t="n">
         <v>59</v>
       </c>
-      <c r="B60" s="18" t="inlineStr">
-        <is>
-          <t>Ί</t>
-        </is>
-      </c>
-      <c r="C60" s="18" t="inlineStr">
-        <is>
-          <t>τόνοι κεφ.</t>
-        </is>
-      </c>
-      <c r="D60" s="14" t="inlineStr">
-        <is>
-          <t>Τονισμένα κεφαλαία φωνήεντα (Ά,Έ,Ή,Ί,Ό,Ύ,Ώ)</t>
+      <c r="B60" s="15" t="inlineStr">
+        <is>
+          <t>φτ</t>
+        </is>
+      </c>
+      <c r="C60" s="16" t="inlineStr">
+        <is>
+          <t>συμφωνικές ομάδες</t>
+        </is>
+      </c>
+      <c r="D60" s="17" t="inlineStr">
+        <is>
+          <t>φτ — π.χ. φτωχός, φτάνω</t>
         </is>
       </c>
     </row>
     <row r="61" ht="18" customHeight="1">
-      <c r="A61" s="17" t="n">
+      <c r="A61" s="20" t="n">
         <v>60</v>
       </c>
-      <c r="B61" s="18" t="inlineStr">
-        <is>
-          <t>Ό</t>
-        </is>
-      </c>
-      <c r="C61" s="18" t="inlineStr">
-        <is>
-          <t>τόνοι κεφ.</t>
-        </is>
-      </c>
-      <c r="D61" s="14" t="inlineStr">
-        <is>
-          <t>Τονισμένα κεφαλαία φωνήεντα (Ά,Έ,Ή,Ί,Ό,Ύ,Ώ)</t>
+      <c r="B61" s="15" t="inlineStr">
+        <is>
+          <t>χτ</t>
+        </is>
+      </c>
+      <c r="C61" s="16" t="inlineStr">
+        <is>
+          <t>συμφωνικές ομάδες</t>
+        </is>
+      </c>
+      <c r="D61" s="17" t="inlineStr">
+        <is>
+          <t>χτ — π.χ. χτες, χτυπώ</t>
         </is>
       </c>
     </row>
     <row r="62" ht="18" customHeight="1">
-      <c r="A62" s="17" t="n">
+      <c r="A62" s="20" t="n">
         <v>61</v>
       </c>
-      <c r="B62" s="18" t="inlineStr">
-        <is>
-          <t>Ύ</t>
-        </is>
-      </c>
-      <c r="C62" s="18" t="inlineStr">
-        <is>
-          <t>τόνοι κεφ.</t>
-        </is>
-      </c>
-      <c r="D62" s="14" t="inlineStr">
-        <is>
-          <t>Τονισμένα κεφαλαία φωνήεντα (Ά,Έ,Ή,Ί,Ό,Ύ,Ώ)</t>
+      <c r="B62" s="15" t="inlineStr">
+        <is>
+          <t>κτ</t>
+        </is>
+      </c>
+      <c r="C62" s="16" t="inlineStr">
+        <is>
+          <t>συμφωνικές ομάδες</t>
+        </is>
+      </c>
+      <c r="D62" s="17" t="inlineStr">
+        <is>
+          <t>κτ — π.χ. κτήριο, κτήνος</t>
         </is>
       </c>
     </row>
     <row r="63" ht="18" customHeight="1">
-      <c r="A63" s="17" t="n">
+      <c r="A63" s="20" t="n">
         <v>62</v>
       </c>
-      <c r="B63" s="18" t="inlineStr">
-        <is>
-          <t>Ώ</t>
-        </is>
-      </c>
-      <c r="C63" s="18" t="inlineStr">
-        <is>
-          <t>τόνοι κεφ.</t>
-        </is>
-      </c>
-      <c r="D63" s="14" t="inlineStr">
-        <is>
-          <t>Τονισμένα κεφαλαία φωνήεντα (Ά,Έ,Ή,Ί,Ό,Ύ,Ώ)</t>
+      <c r="B63" s="15" t="inlineStr">
+        <is>
+          <t>νδ</t>
+        </is>
+      </c>
+      <c r="C63" s="16" t="inlineStr">
+        <is>
+          <t>συμφωνικές ομάδες</t>
+        </is>
+      </c>
+      <c r="D63" s="17" t="inlineStr">
+        <is>
+          <t>νδ — π.χ. άντρας, ένδοξος</t>
         </is>
       </c>
     </row>
     <row r="64" ht="18" customHeight="1">
-      <c r="A64" s="19" t="n">
+      <c r="A64" s="21" t="n">
         <v>63</v>
       </c>
-      <c r="B64" s="20" t="inlineStr">
+      <c r="B64" s="15" t="inlineStr">
         <is>
           <t>αι</t>
         </is>
       </c>
-      <c r="C64" s="20" t="inlineStr">
+      <c r="C64" s="16" t="inlineStr">
         <is>
           <t>δίψηφα</t>
         </is>
       </c>
-      <c r="D64" s="14" t="inlineStr">
-        <is>
-          <t>Δίψηφα σύμφωνα &amp; δίφθογγοι</t>
+      <c r="D64" s="17" t="inlineStr">
+        <is>
+          <t>αι — π.χ. και, παιδί</t>
         </is>
       </c>
     </row>
     <row r="65" ht="18" customHeight="1">
-      <c r="A65" s="19" t="n">
+      <c r="A65" s="21" t="n">
         <v>64</v>
       </c>
-      <c r="B65" s="20" t="inlineStr">
+      <c r="B65" s="15" t="inlineStr">
         <is>
           <t>ει</t>
         </is>
       </c>
-      <c r="C65" s="20" t="inlineStr">
+      <c r="C65" s="16" t="inlineStr">
         <is>
           <t>δίψηφα</t>
         </is>
       </c>
-      <c r="D65" s="14" t="inlineStr">
-        <is>
-          <t>Δίψηφα σύμφωνα &amp; δίφθογγοι</t>
+      <c r="D65" s="17" t="inlineStr">
+        <is>
+          <t>ει — π.χ. είναι, ειρήνη</t>
         </is>
       </c>
     </row>
     <row r="66" ht="18" customHeight="1">
-      <c r="A66" s="19" t="n">
+      <c r="A66" s="21" t="n">
         <v>65</v>
       </c>
-      <c r="B66" s="20" t="inlineStr">
+      <c r="B66" s="15" t="inlineStr">
         <is>
           <t>οι</t>
         </is>
       </c>
-      <c r="C66" s="20" t="inlineStr">
+      <c r="C66" s="16" t="inlineStr">
         <is>
           <t>δίψηφα</t>
         </is>
       </c>
-      <c r="D66" s="14" t="inlineStr">
-        <is>
-          <t>Δίψηφα σύμφωνα &amp; δίφθογγοι</t>
+      <c r="D66" s="17" t="inlineStr">
+        <is>
+          <t>οι — π.χ. οικογένεια</t>
         </is>
       </c>
     </row>
     <row r="67" ht="18" customHeight="1">
-      <c r="A67" s="19" t="n">
+      <c r="A67" s="21" t="n">
         <v>66</v>
       </c>
-      <c r="B67" s="20" t="inlineStr">
+      <c r="B67" s="15" t="inlineStr">
         <is>
           <t>αυ</t>
         </is>
       </c>
-      <c r="C67" s="20" t="inlineStr">
+      <c r="C67" s="16" t="inlineStr">
         <is>
           <t>δίψηφα</t>
         </is>
       </c>
-      <c r="D67" s="14" t="inlineStr">
-        <is>
-          <t>Δίψηφα σύμφωνα &amp; δίφθογγοι</t>
+      <c r="D67" s="17" t="inlineStr">
+        <is>
+          <t>αυ — π.χ. αυτός, αύριο</t>
         </is>
       </c>
     </row>
     <row r="68" ht="18" customHeight="1">
-      <c r="A68" s="19" t="n">
+      <c r="A68" s="21" t="n">
         <v>67</v>
       </c>
-      <c r="B68" s="20" t="inlineStr">
+      <c r="B68" s="15" t="inlineStr">
         <is>
           <t>ευ</t>
         </is>
       </c>
-      <c r="C68" s="20" t="inlineStr">
+      <c r="C68" s="16" t="inlineStr">
         <is>
           <t>δίψηφα</t>
         </is>
       </c>
-      <c r="D68" s="14" t="inlineStr">
-        <is>
-          <t>Δίψηφα σύμφωνα &amp; δίφθογγοι</t>
+      <c r="D68" s="17" t="inlineStr">
+        <is>
+          <t>ευ — π.χ. ευχαριστώ</t>
         </is>
       </c>
     </row>
     <row r="69" ht="18" customHeight="1">
-      <c r="A69" s="19" t="n">
+      <c r="A69" s="21" t="n">
         <v>68</v>
       </c>
-      <c r="B69" s="20" t="inlineStr">
+      <c r="B69" s="15" t="inlineStr">
         <is>
           <t>ου</t>
         </is>
       </c>
-      <c r="C69" s="20" t="inlineStr">
+      <c r="C69" s="16" t="inlineStr">
         <is>
           <t>δίψηφα</t>
         </is>
       </c>
-      <c r="D69" s="14" t="inlineStr">
-        <is>
-          <t>Δίψηφα σύμφωνα &amp; δίφθογγοι</t>
+      <c r="D69" s="17" t="inlineStr">
+        <is>
+          <t>ου — π.χ. ουρανός, ούτε</t>
         </is>
       </c>
     </row>
     <row r="70" ht="18" customHeight="1">
-      <c r="A70" s="19" t="n">
+      <c r="A70" s="21" t="n">
         <v>69</v>
       </c>
-      <c r="B70" s="20" t="inlineStr">
+      <c r="B70" s="15" t="inlineStr">
         <is>
           <t>μπ</t>
         </is>
       </c>
-      <c r="C70" s="20" t="inlineStr">
+      <c r="C70" s="16" t="inlineStr">
         <is>
           <t>δίψηφα</t>
         </is>
       </c>
-      <c r="D70" s="14" t="inlineStr">
-        <is>
-          <t>Δίψηφα σύμφωνα &amp; δίφθογγοι</t>
+      <c r="D70" s="17" t="inlineStr">
+        <is>
+          <t>μπ — π.χ. μπαμπάς, μπλε</t>
         </is>
       </c>
     </row>
     <row r="71" ht="18" customHeight="1">
-      <c r="A71" s="19" t="n">
+      <c r="A71" s="21" t="n">
         <v>70</v>
       </c>
-      <c r="B71" s="20" t="inlineStr">
+      <c r="B71" s="15" t="inlineStr">
         <is>
           <t>ντ</t>
         </is>
       </c>
-      <c r="C71" s="20" t="inlineStr">
+      <c r="C71" s="16" t="inlineStr">
         <is>
           <t>δίψηφα</t>
         </is>
       </c>
-      <c r="D71" s="14" t="inlineStr">
-        <is>
-          <t>Δίψηφα σύμφωνα &amp; δίφθογγοι</t>
+      <c r="D71" s="17" t="inlineStr">
+        <is>
+          <t>ντ — π.χ. ντομάτα, ντύνω</t>
         </is>
       </c>
     </row>
     <row r="72" ht="18" customHeight="1">
-      <c r="A72" s="19" t="n">
+      <c r="A72" s="21" t="n">
         <v>71</v>
       </c>
-      <c r="B72" s="20" t="inlineStr">
+      <c r="B72" s="15" t="inlineStr">
         <is>
           <t>γκ</t>
         </is>
       </c>
-      <c r="C72" s="20" t="inlineStr">
+      <c r="C72" s="16" t="inlineStr">
         <is>
           <t>δίψηφα</t>
         </is>
       </c>
-      <c r="D72" s="14" t="inlineStr">
-        <is>
-          <t>Δίψηφα σύμφωνα &amp; δίφθογγοι</t>
+      <c r="D72" s="17" t="inlineStr">
+        <is>
+          <t>γκ — π.χ. γκαρσόν</t>
         </is>
       </c>
     </row>
     <row r="73" ht="18" customHeight="1">
-      <c r="A73" s="19" t="n">
+      <c r="A73" s="21" t="n">
         <v>72</v>
       </c>
-      <c r="B73" s="20" t="inlineStr">
+      <c r="B73" s="15" t="inlineStr">
         <is>
           <t>τσ</t>
         </is>
       </c>
-      <c r="C73" s="20" t="inlineStr">
+      <c r="C73" s="16" t="inlineStr">
         <is>
           <t>δίψηφα</t>
         </is>
       </c>
-      <c r="D73" s="14" t="inlineStr">
-        <is>
-          <t>Δίψηφα σύμφωνα &amp; δίφθογγοι</t>
+      <c r="D73" s="17" t="inlineStr">
+        <is>
+          <t>τσ — π.χ. τσάντα, τσάι</t>
         </is>
       </c>
     </row>
     <row r="74" ht="18" customHeight="1">
-      <c r="A74" s="19" t="n">
+      <c r="A74" s="21" t="n">
         <v>73</v>
       </c>
-      <c r="B74" s="20" t="inlineStr">
+      <c r="B74" s="15" t="inlineStr">
         <is>
           <t>στ</t>
         </is>
       </c>
-      <c r="C74" s="20" t="inlineStr">
+      <c r="C74" s="16" t="inlineStr">
         <is>
           <t>δίψηφα</t>
         </is>
       </c>
-      <c r="D74" s="14" t="inlineStr">
-        <is>
-          <t>Δίψηφα σύμφωνα &amp; δίφθογγοι</t>
+      <c r="D74" s="17" t="inlineStr">
+        <is>
+          <t>στ — π.χ. στόμα, στρατός</t>
         </is>
       </c>
     </row>
     <row r="75" ht="18" customHeight="1">
-      <c r="A75" s="19" t="n">
+      <c r="A75" s="21" t="n">
         <v>74</v>
       </c>
-      <c r="B75" s="20" t="inlineStr">
+      <c r="B75" s="15" t="inlineStr">
         <is>
           <t>σκ</t>
         </is>
       </c>
-      <c r="C75" s="20" t="inlineStr">
+      <c r="C75" s="16" t="inlineStr">
         <is>
           <t>δίψηφα</t>
         </is>
       </c>
-      <c r="D75" s="14" t="inlineStr">
-        <is>
-          <t>Δίψηφα σύμφωνα &amp; δίφθογγοι</t>
+      <c r="D75" s="17" t="inlineStr">
+        <is>
+          <t>σκ — π.χ. σκύλος, σκιά</t>
         </is>
       </c>
     </row>
     <row r="76" ht="18" customHeight="1">
-      <c r="A76" s="19" t="n">
+      <c r="A76" s="21" t="n">
         <v>75</v>
       </c>
-      <c r="B76" s="20" t="inlineStr">
+      <c r="B76" s="15" t="inlineStr">
         <is>
           <t>πρ</t>
         </is>
       </c>
-      <c r="C76" s="20" t="inlineStr">
+      <c r="C76" s="16" t="inlineStr">
         <is>
           <t>δίψηφα</t>
         </is>
       </c>
-      <c r="D76" s="14" t="inlineStr">
-        <is>
-          <t>Δίψηφα σύμφωνα &amp; δίφθογγοι</t>
+      <c r="D76" s="17" t="inlineStr">
+        <is>
+          <t>πρ — π.χ. πρώτος, πρόσωπο</t>
         </is>
       </c>
     </row>
     <row r="77" ht="18" customHeight="1">
-      <c r="A77" s="19" t="n">
+      <c r="A77" s="21" t="n">
         <v>76</v>
       </c>
-      <c r="B77" s="20" t="inlineStr">
+      <c r="B77" s="15" t="inlineStr">
         <is>
           <t>τρ</t>
         </is>
       </c>
-      <c r="C77" s="20" t="inlineStr">
+      <c r="C77" s="16" t="inlineStr">
         <is>
           <t>δίψηφα</t>
         </is>
       </c>
-      <c r="D77" s="14" t="inlineStr">
-        <is>
-          <t>Δίψηφα σύμφωνα &amp; δίφθογγοι</t>
+      <c r="D77" s="17" t="inlineStr">
+        <is>
+          <t>τρ — π.χ. τρέχω, τρίτος</t>
         </is>
       </c>
     </row>
     <row r="78" ht="18" customHeight="1">
-      <c r="A78" s="19" t="n">
+      <c r="A78" s="21" t="n">
         <v>77</v>
       </c>
-      <c r="B78" s="20" t="inlineStr">
+      <c r="B78" s="15" t="inlineStr">
         <is>
           <t>θρ</t>
         </is>
       </c>
-      <c r="C78" s="20" t="inlineStr">
+      <c r="C78" s="16" t="inlineStr">
         <is>
           <t>δίψηφα</t>
         </is>
       </c>
-      <c r="D78" s="14" t="inlineStr">
-        <is>
-          <t>Δίψηφα σύμφωνα &amp; δίφθογγοι</t>
+      <c r="D78" s="17" t="inlineStr">
+        <is>
+          <t>θρ — π.χ. θρόνος, θρύλος</t>
         </is>
       </c>
     </row>
     <row r="79" ht="18" customHeight="1">
-      <c r="A79" s="19" t="n">
+      <c r="A79" s="21" t="n">
         <v>78</v>
       </c>
-      <c r="B79" s="20" t="inlineStr">
+      <c r="B79" s="15" t="inlineStr">
         <is>
           <t>χρ</t>
         </is>
       </c>
-      <c r="C79" s="20" t="inlineStr">
+      <c r="C79" s="16" t="inlineStr">
         <is>
           <t>δίψηφα</t>
         </is>
       </c>
-      <c r="D79" s="14" t="inlineStr">
-        <is>
-          <t>Δίψηφα σύμφωνα &amp; δίφθογγοι</t>
+      <c r="D79" s="17" t="inlineStr">
+        <is>
+          <t>χρ — π.χ. χρόνος, χρώμα</t>
         </is>
       </c>
     </row>
     <row r="80" ht="18" customHeight="1">
-      <c r="A80" s="19" t="n">
+      <c r="A80" s="21" t="n">
         <v>79</v>
       </c>
-      <c r="B80" s="20" t="inlineStr">
+      <c r="B80" s="15" t="inlineStr">
         <is>
           <t>σπ</t>
         </is>
       </c>
-      <c r="C80" s="20" t="inlineStr">
+      <c r="C80" s="16" t="inlineStr">
         <is>
           <t>δίψηφα</t>
         </is>
       </c>
-      <c r="D80" s="14" t="inlineStr">
-        <is>
-          <t>Δίψηφα σύμφωνα &amp; δίφθογγοι</t>
+      <c r="D80" s="17" t="inlineStr">
+        <is>
+          <t>σπ — π.χ. σπίτι, σπόρος</t>
         </is>
       </c>
     </row>
     <row r="81" ht="18" customHeight="1">
-      <c r="A81" s="19" t="n">
+      <c r="A81" s="21" t="n">
         <v>80</v>
       </c>
-      <c r="B81" s="20" t="inlineStr">
+      <c r="B81" s="15" t="inlineStr">
         <is>
           <t>λλ</t>
         </is>
       </c>
-      <c r="C81" s="20" t="inlineStr">
+      <c r="C81" s="16" t="inlineStr">
         <is>
           <t>δίψηφα</t>
         </is>
       </c>
-      <c r="D81" s="14" t="inlineStr">
-        <is>
-          <t>Δίψηφα σύμφωνα &amp; δίφθογγοι</t>
+      <c r="D81" s="17" t="inlineStr">
+        <is>
+          <t>λλ — π.χ. αλλά, θάλλω</t>
         </is>
       </c>
     </row>

</xml_diff>